<commit_message>
formula updated by MTA
</commit_message>
<xml_diff>
--- a/Required weights.xlsx
+++ b/Required weights.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uofwaterloo-my.sharepoint.com/personal/maraji_uwaterloo_ca/Documents/Symbiosis Lab/Waqas/Side Projects/Bipartitie_3_way/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="554" documentId="13_ncr:1_{C4DF0E6E-FA3F-6D49-AAC4-27CBAFD82E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C8B3788-BE81-A040-B594-5959A5A57997}"/>
+  <xr:revisionPtr revIDLastSave="810" documentId="13_ncr:1_{C4DF0E6E-FA3F-6D49-AAC4-27CBAFD82E60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65C7CE55-5EDA-4748-BABA-19A692D6A587}"/>
   <bookViews>
-    <workbookView xWindow="-1940" yWindow="-19040" windowWidth="24080" windowHeight="17500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8160" yWindow="22740" windowWidth="30240" windowHeight="17480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Relationship Matrix" sheetId="7" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="82">
   <si>
     <t>Communication</t>
   </si>
@@ -251,6 +251,39 @@
   </si>
   <si>
     <t>Visual graphics</t>
+  </si>
+  <si>
+    <t>connections score</t>
+  </si>
+  <si>
+    <t>0.25 * conn score</t>
+  </si>
+  <si>
+    <t>colW</t>
+  </si>
+  <si>
+    <t>CatW</t>
+  </si>
+  <si>
+    <t>0.75*(colW+CatW)</t>
+  </si>
+  <si>
+    <t>Impact score</t>
+  </si>
+  <si>
+    <t>medium conn (left to mid)</t>
+  </si>
+  <si>
+    <t>medium conn (mid to right)</t>
+  </si>
+  <si>
+    <t>strong Conn (left to mid)</t>
+  </si>
+  <si>
+    <t>strong Conn (mid to right)</t>
+  </si>
+  <si>
+    <t>RANK</t>
   </si>
 </sst>
 </file>
@@ -415,7 +448,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -454,8 +487,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="31">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -847,11 +892,51 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1128,13 +1213,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1144,43 +1241,101 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="12">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1541,13 +1696,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C516A866-194E-4597-9029-A5AD387CCDD1}">
-  <dimension ref="B3:AA21"/>
+  <dimension ref="B3:AA32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8.83203125" style="1"/>
     <col min="2" max="2" width="5" style="1" customWidth="1"/>
     <col min="3" max="3" width="24.33203125" style="1" customWidth="1"/>
-    <col min="4" max="18" width="4.1640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="6.1640625" style="1" customWidth="1"/>
+    <col min="5" max="8" width="4.1640625" style="1" customWidth="1"/>
+    <col min="9" max="9" width="7.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="18" width="4.1640625" style="1" customWidth="1"/>
     <col min="19" max="19" width="18.6640625" style="1" customWidth="1"/>
     <col min="23" max="24" width="8.83203125" style="1"/>
     <col min="25" max="25" width="4.1640625" style="1" customWidth="1"/>
@@ -1560,35 +1718,35 @@
   <sheetData>
     <row r="3" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="4" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="109"/>
-      <c r="C4" s="110"/>
-      <c r="D4" s="101" t="s">
+      <c r="B4" s="101"/>
+      <c r="C4" s="102"/>
+      <c r="D4" s="105" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="102"/>
-      <c r="F4" s="102"/>
-      <c r="G4" s="103"/>
-      <c r="H4" s="101" t="s">
+      <c r="E4" s="106"/>
+      <c r="F4" s="106"/>
+      <c r="G4" s="107"/>
+      <c r="H4" s="105" t="s">
         <v>27</v>
       </c>
-      <c r="I4" s="102"/>
-      <c r="J4" s="102"/>
-      <c r="K4" s="103"/>
-      <c r="L4" s="101" t="s">
+      <c r="I4" s="106"/>
+      <c r="J4" s="106"/>
+      <c r="K4" s="107"/>
+      <c r="L4" s="105" t="s">
         <v>28</v>
       </c>
-      <c r="M4" s="102"/>
-      <c r="N4" s="103"/>
-      <c r="O4" s="101" t="s">
+      <c r="M4" s="106"/>
+      <c r="N4" s="107"/>
+      <c r="O4" s="105" t="s">
         <v>29</v>
       </c>
-      <c r="P4" s="102"/>
-      <c r="Q4" s="102"/>
-      <c r="R4" s="103"/>
+      <c r="P4" s="106"/>
+      <c r="Q4" s="106"/>
+      <c r="R4" s="107"/>
     </row>
     <row r="5" spans="2:27" ht="139.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="111"/>
-      <c r="C5" s="112"/>
+      <c r="B5" s="103"/>
+      <c r="C5" s="104"/>
       <c r="D5" s="12" t="s">
         <v>7</v>
       </c>
@@ -1643,7 +1801,7 @@
       <c r="U5" s="88"/>
     </row>
     <row r="6" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="106" t="s">
+      <c r="B6" s="98" t="s">
         <v>1</v>
       </c>
       <c r="C6" s="15" t="s">
@@ -1694,7 +1852,7 @@
       <c r="R6" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="S6" s="104">
+      <c r="S6" s="111">
         <v>10</v>
       </c>
       <c r="T6">
@@ -1702,7 +1860,7 @@
       </c>
     </row>
     <row r="7" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="113"/>
+      <c r="B7" s="108"/>
       <c r="C7" s="23" t="s">
         <v>2</v>
       </c>
@@ -1751,13 +1909,13 @@
       <c r="R7" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="S7" s="104"/>
+      <c r="S7" s="111"/>
       <c r="T7">
         <v>30</v>
       </c>
     </row>
     <row r="8" spans="2:27" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="114"/>
+      <c r="B8" s="109"/>
       <c r="C8" s="35" t="s">
         <v>33</v>
       </c>
@@ -1806,7 +1964,7 @@
       <c r="R8" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="S8" s="104"/>
+      <c r="S8" s="111"/>
       <c r="T8">
         <v>50</v>
       </c>
@@ -1816,7 +1974,7 @@
       <c r="AA8" s="69"/>
     </row>
     <row r="9" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="106" t="s">
+      <c r="B9" s="98" t="s">
         <v>3</v>
       </c>
       <c r="C9" s="15" t="s">
@@ -1867,7 +2025,7 @@
       <c r="R9" s="43" t="s">
         <v>26</v>
       </c>
-      <c r="S9" s="104">
+      <c r="S9" s="111">
         <v>50</v>
       </c>
       <c r="T9">
@@ -1879,7 +2037,7 @@
       <c r="AA9" s="71"/>
     </row>
     <row r="10" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="113"/>
+      <c r="B10" s="108"/>
       <c r="C10" s="23" t="s">
         <v>34</v>
       </c>
@@ -1928,7 +2086,7 @@
       <c r="R10" s="27" t="s">
         <v>26</v>
       </c>
-      <c r="S10" s="104"/>
+      <c r="S10" s="111"/>
       <c r="T10">
         <v>35</v>
       </c>
@@ -1938,7 +2096,7 @@
       <c r="AA10" s="73"/>
     </row>
     <row r="11" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="113"/>
+      <c r="B11" s="108"/>
       <c r="C11" s="23" t="s">
         <v>35</v>
       </c>
@@ -1987,7 +2145,7 @@
       <c r="R11" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="S11" s="104"/>
+      <c r="S11" s="111"/>
       <c r="T11">
         <v>40</v>
       </c>
@@ -1997,7 +2155,7 @@
       <c r="AA11" s="75"/>
     </row>
     <row r="12" spans="2:27" ht="22" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="114"/>
+      <c r="B12" s="109"/>
       <c r="C12" s="35" t="s">
         <v>36</v>
       </c>
@@ -2046,13 +2204,13 @@
       <c r="R12" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="S12" s="104"/>
+      <c r="S12" s="111"/>
       <c r="T12">
         <v>5</v>
       </c>
     </row>
     <row r="13" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="106" t="s">
+      <c r="B13" s="98" t="s">
         <v>5</v>
       </c>
       <c r="C13" s="15" t="s">
@@ -2103,7 +2261,7 @@
       <c r="R13" s="47" t="s">
         <v>25</v>
       </c>
-      <c r="S13" s="104">
+      <c r="S13" s="111">
         <v>25</v>
       </c>
       <c r="T13">
@@ -2118,7 +2276,7 @@
       </c>
     </row>
     <row r="14" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="113"/>
+      <c r="B14" s="108"/>
       <c r="C14" s="23" t="s">
         <v>38</v>
       </c>
@@ -2167,7 +2325,7 @@
       <c r="R14" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="S14" s="104"/>
+      <c r="S14" s="111"/>
       <c r="T14">
         <v>40</v>
       </c>
@@ -2180,7 +2338,7 @@
       </c>
     </row>
     <row r="15" spans="2:27" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="113"/>
+      <c r="B15" s="108"/>
       <c r="C15" s="23" t="s">
         <v>39</v>
       </c>
@@ -2229,7 +2387,7 @@
       <c r="R15" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="S15" s="104"/>
+      <c r="S15" s="111"/>
       <c r="T15">
         <v>25</v>
       </c>
@@ -2242,7 +2400,7 @@
       </c>
     </row>
     <row r="16" spans="2:27" ht="18" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="115"/>
+      <c r="B16" s="110"/>
       <c r="C16" s="48" t="s">
         <v>8</v>
       </c>
@@ -2291,13 +2449,13 @@
       <c r="R16" s="55" t="s">
         <v>24</v>
       </c>
-      <c r="S16" s="104"/>
+      <c r="S16" s="111"/>
       <c r="T16">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="2:20" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="106" t="s">
+      <c r="B17" s="98" t="s">
         <v>0</v>
       </c>
       <c r="C17" s="15" t="s">
@@ -2348,7 +2506,7 @@
       <c r="R17" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="S17" s="104">
+      <c r="S17" s="111">
         <v>15</v>
       </c>
       <c r="T17">
@@ -2356,7 +2514,7 @@
       </c>
     </row>
     <row r="18" spans="2:20" ht="22" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="107"/>
+      <c r="B18" s="99"/>
       <c r="C18" s="23" t="s">
         <v>70</v>
       </c>
@@ -2405,13 +2563,13 @@
       <c r="R18" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="S18" s="104"/>
+      <c r="S18" s="111"/>
       <c r="T18">
         <v>45</v>
       </c>
     </row>
     <row r="19" spans="2:20" ht="17" x14ac:dyDescent="0.2">
-      <c r="B19" s="107"/>
+      <c r="B19" s="99"/>
       <c r="C19" s="57" t="s">
         <v>18</v>
       </c>
@@ -2460,13 +2618,13 @@
       <c r="R19" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="S19" s="104"/>
+      <c r="S19" s="111"/>
       <c r="T19">
         <v>15</v>
       </c>
     </row>
     <row r="20" spans="2:20" ht="28" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="108"/>
+      <c r="B20" s="100"/>
       <c r="C20" s="58" t="s">
         <v>19</v>
       </c>
@@ -2515,7 +2673,7 @@
       <c r="R20" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="S20" s="104"/>
+      <c r="S20" s="111"/>
       <c r="T20">
         <v>10</v>
       </c>
@@ -2524,32 +2682,759 @@
       <c r="C21" s="81" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="105">
+      <c r="D21" s="112">
+        <f>mid2right!C9</f>
+        <v>20</v>
+      </c>
+      <c r="E21" s="112"/>
+      <c r="F21" s="112"/>
+      <c r="G21" s="112"/>
+      <c r="H21" s="132">
+        <f>mid2right!G9</f>
         <v>40</v>
       </c>
-      <c r="E21" s="105"/>
-      <c r="F21" s="105"/>
-      <c r="G21" s="105"/>
-      <c r="H21" s="105">
+      <c r="I21" s="133"/>
+      <c r="J21" s="133"/>
+      <c r="K21" s="134"/>
+      <c r="L21" s="112">
+        <f>mid2right!K9</f>
+        <v>25</v>
+      </c>
+      <c r="M21" s="112"/>
+      <c r="N21" s="112"/>
+      <c r="O21" s="132">
+        <f>mid2right!N9</f>
+        <v>15</v>
+      </c>
+      <c r="P21" s="133"/>
+      <c r="Q21" s="133"/>
+      <c r="R21" s="134"/>
+    </row>
+    <row r="22" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C22" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D22" s="116">
+        <f t="shared" ref="D22:H22" si="0">COUNTIF(D6:D20,"S")</f>
+        <v>1</v>
+      </c>
+      <c r="E22" s="116">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="F22" s="116">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="G22" s="116">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H22" s="120">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="I22" s="121">
+        <f>COUNTIF(I6:I20,"S")</f>
+        <v>10</v>
+      </c>
+      <c r="J22" s="121">
+        <f t="shared" ref="J22:R22" si="1">COUNTIF(J6:J20,"S")</f>
+        <v>2</v>
+      </c>
+      <c r="K22" s="122">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="L22" s="116">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="M22" s="116">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="N22" s="116">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="O22" s="120">
+        <f t="shared" si="1"/>
+        <v>7</v>
+      </c>
+      <c r="P22" s="121">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="Q22" s="121">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="R22" s="122">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C23" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D23" s="116">
+        <f>COUNTIF(mid2right!C4:C8, "S")*1</f>
+        <v>1</v>
+      </c>
+      <c r="E23" s="116">
+        <f>COUNTIF(mid2right!D4:D8, "S")*1</f>
+        <v>3</v>
+      </c>
+      <c r="F23" s="116">
+        <f>COUNTIF(mid2right!E4:E8, "S")*1</f>
+        <v>1</v>
+      </c>
+      <c r="G23" s="116">
+        <f>COUNTIF(mid2right!F4:F8, "S")*1</f>
+        <v>2</v>
+      </c>
+      <c r="H23" s="120">
+        <f>COUNTIF(mid2right!G4:G8, "S")*1</f>
+        <v>4</v>
+      </c>
+      <c r="I23" s="121">
+        <f>COUNTIF(mid2right!H4:H8, "S")*1</f>
+        <v>4</v>
+      </c>
+      <c r="J23" s="121">
+        <f>COUNTIF(mid2right!I4:I8, "S")*1</f>
+        <v>2</v>
+      </c>
+      <c r="K23" s="122">
+        <f>COUNTIF(mid2right!J4:J8, "S")*1</f>
+        <v>2</v>
+      </c>
+      <c r="L23" s="116">
+        <f>COUNTIF(mid2right!K4:K8, "S")*1</f>
+        <v>1</v>
+      </c>
+      <c r="M23" s="116">
+        <f>COUNTIF(mid2right!L4:L8, "S")*1</f>
+        <v>1</v>
+      </c>
+      <c r="N23" s="116">
+        <f>COUNTIF(mid2right!M4:M8, "S")*1</f>
+        <v>2</v>
+      </c>
+      <c r="O23" s="120">
+        <f>COUNTIF(mid2right!N4:N8, "S")*1</f>
+        <v>3</v>
+      </c>
+      <c r="P23" s="121">
+        <f>COUNTIF(mid2right!O4:O8, "S")*1</f>
+        <v>3</v>
+      </c>
+      <c r="Q23" s="121">
+        <f>COUNTIF(mid2right!P4:P8, "S")*1</f>
+        <v>1</v>
+      </c>
+      <c r="R23" s="122">
+        <f>COUNTIF(mid2right!Q4:Q8, "S")*1</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C24" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D24" s="117">
+        <f>COUNTIF(D6:D20,"M")</f>
+        <v>3</v>
+      </c>
+      <c r="E24" s="117">
+        <f t="shared" ref="E24:R24" si="2">COUNTIF(E6:E20,"M")</f>
+        <v>3</v>
+      </c>
+      <c r="F24" s="117">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="G24" s="117">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="H24" s="123">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+      <c r="I24" s="124">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="J24" s="124">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="K24" s="125">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="L24" s="117">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="M24" s="117">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="N24" s="117">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="O24" s="123">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="P24" s="124">
+        <f t="shared" si="2"/>
+        <v>7</v>
+      </c>
+      <c r="Q24" s="124">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="R24" s="125">
+        <f t="shared" si="2"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C25" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D25" s="117">
+        <f>COUNTIF(mid2right!C4:C8,"M")</f>
+        <v>1</v>
+      </c>
+      <c r="E25" s="117">
+        <f>COUNTIF(mid2right!D4:D8,"M")</f>
+        <v>2</v>
+      </c>
+      <c r="F25" s="117">
+        <f>COUNTIF(mid2right!E4:E8,"M")</f>
+        <v>4</v>
+      </c>
+      <c r="G25" s="117">
+        <f>COUNTIF(mid2right!F4:F8,"M")</f>
+        <v>1</v>
+      </c>
+      <c r="H25" s="123">
+        <f>COUNTIF(mid2right!G4:G8,"M")</f>
+        <v>1</v>
+      </c>
+      <c r="I25" s="124">
+        <f>COUNTIF(mid2right!H4:H8,"M")</f>
+        <v>1</v>
+      </c>
+      <c r="J25" s="124">
+        <f>COUNTIF(mid2right!I4:I8,"M")</f>
+        <v>3</v>
+      </c>
+      <c r="K25" s="125">
+        <f>COUNTIF(mid2right!J4:J8,"M")</f>
+        <v>2</v>
+      </c>
+      <c r="L25" s="117">
+        <f>COUNTIF(mid2right!K4:K8,"M")</f>
+        <v>0</v>
+      </c>
+      <c r="M25" s="117">
+        <f>COUNTIF(mid2right!L4:L8,"M")</f>
+        <v>4</v>
+      </c>
+      <c r="N25" s="117">
+        <f>COUNTIF(mid2right!M4:M8,"M")</f>
+        <v>2</v>
+      </c>
+      <c r="O25" s="123">
+        <f>COUNTIF(mid2right!N4:N8,"M")</f>
+        <v>0</v>
+      </c>
+      <c r="P25" s="124">
+        <f>COUNTIF(mid2right!O4:O8,"M")</f>
+        <v>2</v>
+      </c>
+      <c r="Q25" s="124">
+        <f>COUNTIF(mid2right!P4:P8,"M")</f>
+        <v>0</v>
+      </c>
+      <c r="R25" s="125">
+        <f>COUNTIF(mid2right!Q4:Q8,"M")</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C26" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D26" s="1">
+        <f t="shared" ref="D26:H26" si="3">3*SUM(D22:D23) + SUM(D24:D25)</f>
+        <v>10</v>
+      </c>
+      <c r="E26" s="1">
+        <f t="shared" si="3"/>
+        <v>38</v>
+      </c>
+      <c r="F26" s="1">
+        <f t="shared" si="3"/>
+        <v>20</v>
+      </c>
+      <c r="G26" s="1">
+        <f t="shared" si="3"/>
+        <v>23</v>
+      </c>
+      <c r="H26" s="126">
+        <f t="shared" si="3"/>
+        <v>44</v>
+      </c>
+      <c r="I26" s="127">
+        <f>3*SUM(I22:I23) + SUM(I24:I25)</f>
+        <v>45</v>
+      </c>
+      <c r="J26" s="127">
+        <f t="shared" ref="J26:R26" si="4">3*SUM(J22:J23) + SUM(J24:J25)</f>
+        <v>22</v>
+      </c>
+      <c r="K26" s="128">
+        <f t="shared" si="4"/>
+        <v>24</v>
+      </c>
+      <c r="L26" s="1">
+        <f t="shared" si="4"/>
+        <v>24</v>
+      </c>
+      <c r="M26" s="1">
+        <f t="shared" si="4"/>
         <v>30</v>
       </c>
-      <c r="I21" s="105"/>
-      <c r="J21" s="105"/>
-      <c r="K21" s="105"/>
-      <c r="L21" s="105">
+      <c r="N26" s="1">
+        <f t="shared" si="4"/>
+        <v>33</v>
+      </c>
+      <c r="O26" s="126">
+        <f t="shared" si="4"/>
+        <v>32</v>
+      </c>
+      <c r="P26" s="127">
+        <f t="shared" si="4"/>
+        <v>21</v>
+      </c>
+      <c r="Q26" s="127">
+        <f t="shared" si="4"/>
+        <v>13</v>
+      </c>
+      <c r="R26" s="128">
+        <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="M21" s="105"/>
-      <c r="N21" s="105"/>
-      <c r="O21" s="105">
+    </row>
+    <row r="27" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C27" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D27" s="1">
+        <f t="shared" ref="D27:H27" si="5">0.25*D26</f>
+        <v>2.5</v>
+      </c>
+      <c r="E27" s="1">
+        <f t="shared" si="5"/>
+        <v>9.5</v>
+      </c>
+      <c r="F27" s="1">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="G27" s="1">
+        <f t="shared" si="5"/>
+        <v>5.75</v>
+      </c>
+      <c r="H27" s="126">
+        <f t="shared" si="5"/>
+        <v>11</v>
+      </c>
+      <c r="I27" s="127">
+        <f>0.25*I26</f>
+        <v>11.25</v>
+      </c>
+      <c r="J27" s="127">
+        <f t="shared" ref="J27:R27" si="6">0.25*J26</f>
+        <v>5.5</v>
+      </c>
+      <c r="K27" s="128">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="L27" s="1">
+        <f t="shared" si="6"/>
+        <v>6</v>
+      </c>
+      <c r="M27" s="1">
+        <f t="shared" si="6"/>
+        <v>7.5</v>
+      </c>
+      <c r="N27" s="1">
+        <f t="shared" si="6"/>
+        <v>8.25</v>
+      </c>
+      <c r="O27" s="126">
+        <f t="shared" si="6"/>
+        <v>8</v>
+      </c>
+      <c r="P27" s="127">
+        <f t="shared" si="6"/>
+        <v>5.25</v>
+      </c>
+      <c r="Q27" s="127">
+        <f t="shared" si="6"/>
+        <v>3.25</v>
+      </c>
+      <c r="R27" s="128">
+        <f t="shared" si="6"/>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C28" s="118" t="s">
+        <v>73</v>
+      </c>
+      <c r="D28" s="118">
+        <f>mid2right!C10*mid2right!C9/100</f>
+        <v>4</v>
+      </c>
+      <c r="E28" s="118">
+        <f>mid2right!D10*mid2right!C9/100</f>
+        <v>6</v>
+      </c>
+      <c r="F28" s="118">
+        <f>mid2right!E10*mid2right!C9/100</f>
+        <v>3</v>
+      </c>
+      <c r="G28" s="118">
+        <f>mid2right!F10*mid2right!C9/100</f>
+        <v>7</v>
+      </c>
+      <c r="H28" s="129">
+        <f>mid2right!G10*mid2right!G9/100</f>
         <v>10</v>
       </c>
-      <c r="P21" s="105"/>
-      <c r="Q21" s="105"/>
-      <c r="R21" s="105"/>
+      <c r="I28" s="130">
+        <f>mid2right!H10*mid2right!G9/100</f>
+        <v>12</v>
+      </c>
+      <c r="J28" s="130">
+        <f>mid2right!I10*mid2right!G9/100</f>
+        <v>12</v>
+      </c>
+      <c r="K28" s="131">
+        <f>mid2right!J10*mid2right!G9/100</f>
+        <v>6</v>
+      </c>
+      <c r="L28" s="118">
+        <f>mid2right!K10*mid2right!K9/100</f>
+        <v>7.5</v>
+      </c>
+      <c r="M28" s="118">
+        <f>mid2right!L10*mid2right!K9/100</f>
+        <v>7.5</v>
+      </c>
+      <c r="N28" s="118">
+        <f>mid2right!M10*mid2right!K9/100</f>
+        <v>10</v>
+      </c>
+      <c r="O28" s="129">
+        <f>mid2right!N10*mid2right!N9/100</f>
+        <v>5.25</v>
+      </c>
+      <c r="P28" s="130">
+        <f>mid2right!O10*mid2right!N9/100</f>
+        <v>3.75</v>
+      </c>
+      <c r="Q28" s="130">
+        <f>mid2right!P10*mid2right!N9/100</f>
+        <v>3.75</v>
+      </c>
+      <c r="R28" s="131">
+        <f>mid2right!Q10*mid2right!N9/100</f>
+        <v>2.25</v>
+      </c>
+    </row>
+    <row r="29" spans="2:20" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="C29" s="118" t="s">
+        <v>74</v>
+      </c>
+      <c r="D29" s="118">
+        <f>mid2right!C10</f>
+        <v>20</v>
+      </c>
+      <c r="E29" s="118">
+        <f>mid2right!D10</f>
+        <v>30</v>
+      </c>
+      <c r="F29" s="118">
+        <f>mid2right!E10</f>
+        <v>15</v>
+      </c>
+      <c r="G29" s="118">
+        <f>mid2right!F10</f>
+        <v>35</v>
+      </c>
+      <c r="H29" s="135">
+        <f>mid2right!G10</f>
+        <v>25</v>
+      </c>
+      <c r="I29" s="136">
+        <f>mid2right!H10</f>
+        <v>30</v>
+      </c>
+      <c r="J29" s="136">
+        <f>mid2right!I10</f>
+        <v>30</v>
+      </c>
+      <c r="K29" s="137">
+        <f>mid2right!J10</f>
+        <v>15</v>
+      </c>
+      <c r="L29" s="118">
+        <f>mid2right!K10</f>
+        <v>30</v>
+      </c>
+      <c r="M29" s="118">
+        <f>mid2right!L10</f>
+        <v>30</v>
+      </c>
+      <c r="N29" s="118">
+        <f>mid2right!M10</f>
+        <v>40</v>
+      </c>
+      <c r="O29" s="135">
+        <f>mid2right!N10</f>
+        <v>35</v>
+      </c>
+      <c r="P29" s="136">
+        <f>mid2right!O10</f>
+        <v>25</v>
+      </c>
+      <c r="Q29" s="136">
+        <f>mid2right!P10</f>
+        <v>25</v>
+      </c>
+      <c r="R29" s="137">
+        <f>mid2right!Q10</f>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C30" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D30" s="1">
+        <f>0.75*D28*D29</f>
+        <v>60</v>
+      </c>
+      <c r="E30" s="1">
+        <f t="shared" ref="E30:R30" si="7">0.75*E28*E29</f>
+        <v>135</v>
+      </c>
+      <c r="F30" s="1">
+        <f t="shared" si="7"/>
+        <v>33.75</v>
+      </c>
+      <c r="G30" s="1">
+        <f t="shared" si="7"/>
+        <v>183.75</v>
+      </c>
+      <c r="H30" s="1">
+        <f t="shared" si="7"/>
+        <v>187.5</v>
+      </c>
+      <c r="I30" s="1">
+        <f t="shared" si="7"/>
+        <v>270</v>
+      </c>
+      <c r="J30" s="1">
+        <f t="shared" si="7"/>
+        <v>270</v>
+      </c>
+      <c r="K30" s="1">
+        <f t="shared" si="7"/>
+        <v>67.5</v>
+      </c>
+      <c r="L30" s="1">
+        <f t="shared" si="7"/>
+        <v>168.75</v>
+      </c>
+      <c r="M30" s="1">
+        <f t="shared" si="7"/>
+        <v>168.75</v>
+      </c>
+      <c r="N30" s="1">
+        <f t="shared" si="7"/>
+        <v>300</v>
+      </c>
+      <c r="O30" s="1">
+        <f t="shared" si="7"/>
+        <v>137.8125</v>
+      </c>
+      <c r="P30" s="1">
+        <f t="shared" si="7"/>
+        <v>70.3125</v>
+      </c>
+      <c r="Q30" s="1">
+        <f t="shared" si="7"/>
+        <v>70.3125</v>
+      </c>
+      <c r="R30" s="1">
+        <f t="shared" si="7"/>
+        <v>25.3125</v>
+      </c>
+    </row>
+    <row r="31" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C31" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="1">
+        <f t="shared" ref="D31:H31" si="8">D30+D27</f>
+        <v>62.5</v>
+      </c>
+      <c r="E31" s="1">
+        <f t="shared" si="8"/>
+        <v>144.5</v>
+      </c>
+      <c r="F31" s="1">
+        <f t="shared" si="8"/>
+        <v>38.75</v>
+      </c>
+      <c r="G31" s="1">
+        <f t="shared" si="8"/>
+        <v>189.5</v>
+      </c>
+      <c r="H31" s="1">
+        <f t="shared" si="8"/>
+        <v>198.5</v>
+      </c>
+      <c r="I31" s="1">
+        <f>I30+I27</f>
+        <v>281.25</v>
+      </c>
+      <c r="J31" s="1">
+        <f t="shared" ref="J31:R31" si="9">J30+J27</f>
+        <v>275.5</v>
+      </c>
+      <c r="K31" s="1">
+        <f t="shared" si="9"/>
+        <v>73.5</v>
+      </c>
+      <c r="L31" s="1">
+        <f t="shared" si="9"/>
+        <v>174.75</v>
+      </c>
+      <c r="M31" s="1">
+        <f t="shared" si="9"/>
+        <v>176.25</v>
+      </c>
+      <c r="N31" s="1">
+        <f t="shared" si="9"/>
+        <v>308.25</v>
+      </c>
+      <c r="O31" s="1">
+        <f t="shared" si="9"/>
+        <v>145.8125</v>
+      </c>
+      <c r="P31" s="1">
+        <f t="shared" si="9"/>
+        <v>75.5625</v>
+      </c>
+      <c r="Q31" s="1">
+        <f t="shared" si="9"/>
+        <v>73.5625</v>
+      </c>
+      <c r="R31" s="1">
+        <f t="shared" si="9"/>
+        <v>30.3125</v>
+      </c>
+    </row>
+    <row r="32" spans="2:20" x14ac:dyDescent="0.2">
+      <c r="C32" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D32" s="1">
+        <f>_xlfn.RANK.EQ(D31,$D$31:$R$31)</f>
+        <v>13</v>
+      </c>
+      <c r="E32" s="1">
+        <f t="shared" ref="E32:R32" si="10">_xlfn.RANK.EQ(E31,$D$31:$R$31)</f>
+        <v>9</v>
+      </c>
+      <c r="F32" s="1">
+        <f t="shared" si="10"/>
+        <v>14</v>
+      </c>
+      <c r="G32" s="1">
+        <f t="shared" si="10"/>
+        <v>5</v>
+      </c>
+      <c r="H32" s="1">
+        <f t="shared" si="10"/>
+        <v>4</v>
+      </c>
+      <c r="I32" s="1">
+        <f t="shared" si="10"/>
+        <v>2</v>
+      </c>
+      <c r="J32" s="1">
+        <f t="shared" si="10"/>
+        <v>3</v>
+      </c>
+      <c r="K32" s="1">
+        <f t="shared" si="10"/>
+        <v>12</v>
+      </c>
+      <c r="L32" s="1">
+        <f t="shared" si="10"/>
+        <v>7</v>
+      </c>
+      <c r="M32" s="1">
+        <f t="shared" si="10"/>
+        <v>6</v>
+      </c>
+      <c r="N32" s="1">
+        <f t="shared" si="10"/>
+        <v>1</v>
+      </c>
+      <c r="O32" s="1">
+        <f t="shared" si="10"/>
+        <v>8</v>
+      </c>
+      <c r="P32" s="1">
+        <f t="shared" si="10"/>
+        <v>10</v>
+      </c>
+      <c r="Q32" s="1">
+        <f t="shared" si="10"/>
+        <v>11</v>
+      </c>
+      <c r="R32" s="1">
+        <f t="shared" si="10"/>
+        <v>15</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="S6:S8"/>
+    <mergeCell ref="S9:S12"/>
+    <mergeCell ref="S13:S16"/>
+    <mergeCell ref="S17:S20"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="L21:N21"/>
+    <mergeCell ref="O21:R21"/>
     <mergeCell ref="B17:B20"/>
     <mergeCell ref="B4:C5"/>
     <mergeCell ref="O4:R4"/>
@@ -2559,27 +3444,31 @@
     <mergeCell ref="D4:G4"/>
     <mergeCell ref="H4:K4"/>
     <mergeCell ref="L4:N4"/>
-    <mergeCell ref="S6:S8"/>
-    <mergeCell ref="S9:S12"/>
-    <mergeCell ref="S13:S16"/>
-    <mergeCell ref="S17:S20"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="L21:N21"/>
-    <mergeCell ref="O21:R21"/>
   </mergeCells>
   <conditionalFormatting sqref="D6:R20">
-    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="7" priority="2" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",D6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="6" priority="2" operator="containsText" text="W">
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="W">
       <formula>NOT(ISERROR(SEARCH("W",D6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="S">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="S">
       <formula>NOT(ISERROR(SEARCH("S",D6)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",D6)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D31:R31">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2589,12 +3478,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC40F516-73D9-AF40-BBFA-DA5A09FC7B78}">
-  <dimension ref="A1:R10"/>
+  <dimension ref="A1:R11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2.1640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.1640625" customWidth="1"/>
-    <col min="3" max="17" width="3.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.83203125" customWidth="1"/>
+    <col min="4" max="17" width="3.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="17" thickBot="1" x14ac:dyDescent="0.25">
@@ -2649,29 +3539,29 @@
     <row r="2" spans="1:18" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1"/>
       <c r="B2" s="82"/>
-      <c r="C2" s="101" t="s">
+      <c r="C2" s="105" t="s">
         <v>48</v>
       </c>
-      <c r="D2" s="102"/>
-      <c r="E2" s="102"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="101" t="s">
+      <c r="D2" s="106"/>
+      <c r="E2" s="106"/>
+      <c r="F2" s="107"/>
+      <c r="G2" s="105" t="s">
         <v>27</v>
       </c>
-      <c r="H2" s="102"/>
-      <c r="I2" s="102"/>
-      <c r="J2" s="103"/>
-      <c r="K2" s="101" t="s">
+      <c r="H2" s="106"/>
+      <c r="I2" s="106"/>
+      <c r="J2" s="107"/>
+      <c r="K2" s="105" t="s">
         <v>28</v>
       </c>
-      <c r="L2" s="102"/>
-      <c r="M2" s="103"/>
-      <c r="N2" s="101" t="s">
+      <c r="L2" s="106"/>
+      <c r="M2" s="107"/>
+      <c r="N2" s="105" t="s">
         <v>29</v>
       </c>
-      <c r="O2" s="102"/>
-      <c r="P2" s="102"/>
-      <c r="Q2" s="103"/>
+      <c r="O2" s="106"/>
+      <c r="P2" s="106"/>
+      <c r="Q2" s="107"/>
       <c r="R2" s="80" t="s">
         <v>47</v>
       </c>
@@ -3025,29 +3915,29 @@
       <c r="B9" s="95" t="s">
         <v>47</v>
       </c>
-      <c r="C9" s="98">
+      <c r="C9" s="113">
         <v>20</v>
       </c>
-      <c r="D9" s="99"/>
-      <c r="E9" s="99"/>
-      <c r="F9" s="100"/>
-      <c r="G9" s="98">
+      <c r="D9" s="114"/>
+      <c r="E9" s="114"/>
+      <c r="F9" s="115"/>
+      <c r="G9" s="113">
         <v>40</v>
       </c>
-      <c r="H9" s="99"/>
-      <c r="I9" s="99"/>
-      <c r="J9" s="100"/>
-      <c r="K9" s="98">
-        <v>25</v>
-      </c>
-      <c r="L9" s="99"/>
-      <c r="M9" s="100"/>
-      <c r="N9" s="98">
+      <c r="H9" s="114"/>
+      <c r="I9" s="114"/>
+      <c r="J9" s="115"/>
+      <c r="K9" s="113">
+        <v>25</v>
+      </c>
+      <c r="L9" s="114"/>
+      <c r="M9" s="115"/>
+      <c r="N9" s="113">
         <v>15</v>
       </c>
-      <c r="O9" s="99"/>
-      <c r="P9" s="99"/>
-      <c r="Q9" s="100"/>
+      <c r="O9" s="114"/>
+      <c r="P9" s="114"/>
+      <c r="Q9" s="115"/>
     </row>
     <row r="10" spans="1:18" ht="18" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B10" s="96" t="s">
@@ -3078,13 +3968,13 @@
         <v>15</v>
       </c>
       <c r="K10" s="84">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="L10" s="85">
         <v>30</v>
       </c>
       <c r="M10" s="86">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="N10" s="84">
         <v>35</v>
@@ -3098,6 +3988,9 @@
       <c r="Q10" s="86">
         <v>15</v>
       </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="C11" s="119"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -3111,16 +4004,16 @@
     <mergeCell ref="K2:M2"/>
   </mergeCells>
   <conditionalFormatting sqref="C4:Q8">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="11" priority="1" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",C4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="2" operator="containsText" text="W">
+    <cfRule type="containsText" dxfId="10" priority="2" operator="containsText" text="W">
       <formula>NOT(ISERROR(SEARCH("W",C4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="3" operator="containsText" text="S">
+    <cfRule type="containsText" dxfId="9" priority="3" operator="containsText" text="S">
       <formula>NOT(ISERROR(SEARCH("S",C4)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="4" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="8" priority="4" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",C4)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>